<commit_message>
Updated PLPAD to PLPD
</commit_message>
<xml_diff>
--- a/Data/1999_F105_CO_AGIIS/1999_F105_CO_AGIIS_CropCanopy.xlsx
+++ b/Data/1999_F105_CO_AGIIS/1999_F105_CO_AGIIS_CropCanopy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI project\cottondata\Data\1999_F105_CO_AGIIS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E214FF5A-D013-4B08-8B14-902906393C12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F70D8499-0282-41CD-B252-920C53AA4B90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1665" yWindow="-27285" windowWidth="17820" windowHeight="26805" xr2:uid="{5E62E68C-7E3C-475C-975C-774D7039174E}"/>
+    <workbookView xWindow="-1470" yWindow="-28410" windowWidth="17805" windowHeight="20370" xr2:uid="{5E62E68C-7E3C-475C-975C-774D7039174E}"/>
   </bookViews>
   <sheets>
     <sheet name="Canopy" sheetId="1" r:id="rId1"/>
@@ -22,9 +22,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="425">
   <si>
-    <t>PLPAD</t>
-  </si>
-  <si>
     <t>CHTDcm</t>
   </si>
   <si>
@@ -1295,6 +1292,9 @@
   </si>
   <si>
     <t>CCID</t>
+  </si>
+  <si>
+    <t>PLPD</t>
   </si>
 </sst>
 </file>
@@ -2168,24 +2168,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>423</v>
+      </c>
+      <c r="B1" t="s">
         <v>424</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>2</v>
-      </c>
-      <c r="E1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" s="1">
         <v>9.5</v>
@@ -2202,7 +2202,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B3" s="1">
         <v>10.5</v>
@@ -2219,7 +2219,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" s="1">
         <v>12.5</v>
@@ -2236,7 +2236,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" s="1">
         <v>9</v>
@@ -2253,7 +2253,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" s="1">
         <v>8.5</v>
@@ -2270,7 +2270,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7" s="1">
         <v>12</v>
@@ -2287,7 +2287,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B8" s="1">
         <v>11</v>
@@ -2304,7 +2304,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" s="1">
         <v>8</v>
@@ -2321,7 +2321,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
@@ -2338,7 +2338,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" s="1">
         <v>7.5</v>
@@ -2355,7 +2355,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" s="1">
         <v>6.5</v>
@@ -2372,7 +2372,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B13" s="1">
         <v>9.5</v>
@@ -2389,7 +2389,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14" s="1">
         <v>12</v>
@@ -2406,7 +2406,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15" s="1">
         <v>7.5</v>
@@ -2423,7 +2423,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B16" s="1">
         <v>13.5</v>
@@ -2440,7 +2440,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B17" s="1">
         <v>11.5</v>
@@ -2457,7 +2457,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B18" s="1">
         <v>6.5</v>
@@ -2474,7 +2474,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B19" s="1">
         <v>8</v>
@@ -2491,7 +2491,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B20" s="1">
         <v>12</v>
@@ -2508,7 +2508,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B21" s="1">
         <v>9.5</v>
@@ -2525,7 +2525,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B22" s="1">
         <v>8</v>
@@ -2542,7 +2542,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B23" s="1">
         <v>9</v>
@@ -2559,7 +2559,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B24" s="1">
         <v>9</v>
@@ -2576,7 +2576,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B25" s="1">
         <v>10</v>
@@ -2593,7 +2593,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B26" s="1">
         <v>9.5</v>
@@ -2610,7 +2610,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B27" s="1">
         <v>11</v>
@@ -2627,7 +2627,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B28" s="1">
         <v>13</v>
@@ -2644,7 +2644,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B29" s="1">
         <v>11</v>
@@ -2661,7 +2661,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B30" s="1">
         <v>8.5</v>
@@ -2678,7 +2678,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B31" s="1">
         <v>11.5</v>
@@ -2695,7 +2695,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B32" s="1">
         <v>7.5</v>
@@ -2712,7 +2712,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B33" s="1">
         <v>9.5</v>
@@ -2729,7 +2729,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B34" s="1">
         <v>12.5</v>
@@ -2746,7 +2746,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B35" s="1">
         <v>10</v>
@@ -2763,7 +2763,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B36" s="1">
         <v>9.5</v>
@@ -2780,7 +2780,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B37" s="1">
         <v>13</v>
@@ -2797,7 +2797,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B38" s="1">
         <v>9.5</v>
@@ -2814,7 +2814,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B39" s="1">
         <v>12.5</v>
@@ -2831,7 +2831,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B40" s="1">
         <v>12.5</v>
@@ -2848,7 +2848,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B41" s="1">
         <v>11.5</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B42" s="1">
         <v>12.5</v>
@@ -2882,7 +2882,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B43" s="1">
         <v>11</v>
@@ -2899,7 +2899,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B44" s="1">
         <v>8</v>
@@ -2916,7 +2916,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B45" s="1">
         <v>11.5</v>
@@ -2933,7 +2933,7 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B46" s="1">
         <v>12.5</v>
@@ -2950,7 +2950,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B47" s="1">
         <v>11</v>
@@ -2967,7 +2967,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B48" s="1">
         <v>9</v>
@@ -2984,7 +2984,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B49" s="1">
         <v>12</v>
@@ -3001,7 +3001,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B50" s="1">
         <v>12.5</v>
@@ -3018,7 +3018,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B51" s="1">
         <v>7</v>
@@ -3035,7 +3035,7 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B52" s="1">
         <v>12.5</v>
@@ -3052,7 +3052,7 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B53" s="1">
         <v>12</v>
@@ -3069,7 +3069,7 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B54" s="1">
         <v>4</v>
@@ -3086,7 +3086,7 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B55" s="1">
         <v>11</v>
@@ -3103,7 +3103,7 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B56" s="1">
         <v>10</v>
@@ -3120,7 +3120,7 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B57" s="1">
         <v>10</v>
@@ -3137,7 +3137,7 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B58" s="1">
         <v>8.5</v>
@@ -3154,7 +3154,7 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B59" s="1">
         <v>11</v>
@@ -3171,7 +3171,7 @@
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B60" s="1">
         <v>11</v>
@@ -3188,7 +3188,7 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B61" s="1">
         <v>6.5</v>
@@ -3205,7 +3205,7 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B62" s="1">
         <v>12</v>
@@ -3222,7 +3222,7 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B63" s="1">
         <v>7</v>
@@ -3239,7 +3239,7 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B64" s="1">
         <v>10</v>
@@ -3256,7 +3256,7 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B65" s="1">
         <v>9</v>
@@ -3273,7 +3273,7 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B66" s="1">
         <v>6</v>
@@ -3290,7 +3290,7 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B67" s="1">
         <v>14.5</v>
@@ -3307,7 +3307,7 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B68" s="1">
         <v>12</v>
@@ -3324,7 +3324,7 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B69" s="1">
         <v>10</v>
@@ -3341,7 +3341,7 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B70" s="1">
         <v>10</v>
@@ -3358,7 +3358,7 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B71" s="1">
         <v>11</v>
@@ -3375,7 +3375,7 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B72" s="1">
         <v>5.5</v>
@@ -3392,7 +3392,7 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B73" s="1">
         <v>11</v>
@@ -3409,7 +3409,7 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B74" s="1">
         <v>7</v>
@@ -3426,7 +3426,7 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B75" s="1">
         <v>9.5</v>
@@ -3443,7 +3443,7 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B76" s="1">
         <v>13</v>
@@ -3460,7 +3460,7 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B77" s="1">
         <v>10</v>
@@ -3477,7 +3477,7 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B78" s="1">
         <v>10</v>
@@ -3494,7 +3494,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B79" s="1">
         <v>8.5</v>
@@ -3511,7 +3511,7 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B80" s="1">
         <v>7.5</v>
@@ -3528,7 +3528,7 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B81" s="1">
         <v>9</v>
@@ -3545,7 +3545,7 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B82" s="1">
         <v>10</v>
@@ -3562,7 +3562,7 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B83" s="1">
         <v>11</v>
@@ -3579,7 +3579,7 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B84" s="1">
         <v>8</v>
@@ -3596,7 +3596,7 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B85" s="1">
         <v>8.5</v>
@@ -3613,7 +3613,7 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B86" s="1">
         <v>8.5</v>
@@ -3630,7 +3630,7 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B87" s="1">
         <v>13.5</v>
@@ -3647,7 +3647,7 @@
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B88" s="1">
         <v>11.5</v>
@@ -3664,7 +3664,7 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B89" s="1">
         <v>10</v>
@@ -3681,7 +3681,7 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B90" s="1">
         <v>11</v>
@@ -3698,7 +3698,7 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B91" s="1">
         <v>10</v>
@@ -3715,7 +3715,7 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B92" s="1">
         <v>10</v>
@@ -3732,7 +3732,7 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B93" s="1">
         <v>7</v>
@@ -3749,7 +3749,7 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B94" s="1">
         <v>10</v>
@@ -3766,7 +3766,7 @@
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B95" s="1">
         <v>12.5</v>
@@ -3783,7 +3783,7 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B96" s="1">
         <v>13.5</v>
@@ -3800,7 +3800,7 @@
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B97" s="1">
         <v>8.5</v>
@@ -3817,7 +3817,7 @@
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B98" s="1">
         <v>11.5</v>
@@ -3834,7 +3834,7 @@
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B99" s="1">
         <v>9</v>
@@ -3851,7 +3851,7 @@
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B100" s="1">
         <v>8.5</v>
@@ -3868,7 +3868,7 @@
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B101" s="1">
         <v>7.5</v>
@@ -3885,7 +3885,7 @@
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B102" s="1">
         <v>6</v>
@@ -3902,7 +3902,7 @@
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B103" s="1">
         <v>11</v>
@@ -3919,7 +3919,7 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B104" s="1">
         <v>5</v>
@@ -3936,7 +3936,7 @@
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B105" s="1">
         <v>12</v>
@@ -3953,7 +3953,7 @@
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B106" s="1">
         <v>8.5</v>
@@ -3970,7 +3970,7 @@
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B107" s="1">
         <v>6.5</v>
@@ -3987,7 +3987,7 @@
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B108" s="1">
         <v>8.5</v>
@@ -4004,7 +4004,7 @@
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B109" s="1">
         <v>11</v>
@@ -4021,7 +4021,7 @@
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B110" s="1">
         <v>9.5</v>
@@ -4038,7 +4038,7 @@
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B111" s="1">
         <v>10.5</v>
@@ -4055,7 +4055,7 @@
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B112" s="1">
         <v>9</v>
@@ -4072,7 +4072,7 @@
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B113" s="1">
         <v>10.5</v>
@@ -4089,7 +4089,7 @@
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B114" s="1">
         <v>11.5</v>
@@ -4106,7 +4106,7 @@
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B115" s="1">
         <v>8.5</v>
@@ -4123,7 +4123,7 @@
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B116" s="1">
         <v>8</v>
@@ -4140,7 +4140,7 @@
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B117" s="1">
         <v>11</v>
@@ -4157,7 +4157,7 @@
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B118" s="1">
         <v>8</v>
@@ -4174,7 +4174,7 @@
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B119" s="1">
         <v>8.5</v>
@@ -4191,7 +4191,7 @@
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B120" s="1">
         <v>9.5</v>
@@ -4208,7 +4208,7 @@
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B121" s="1">
         <v>9.5</v>
@@ -4225,7 +4225,7 @@
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B122" s="1">
         <v>10.5</v>
@@ -4242,7 +4242,7 @@
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B123" s="1">
         <v>8</v>
@@ -4259,7 +4259,7 @@
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B124" s="1">
         <v>9</v>
@@ -4276,7 +4276,7 @@
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B125" s="1">
         <v>9.5</v>
@@ -4293,7 +4293,7 @@
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B126" s="1">
         <v>7</v>
@@ -4310,7 +4310,7 @@
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B127" s="1">
         <v>11.5</v>
@@ -4327,7 +4327,7 @@
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B128" s="1">
         <v>8</v>
@@ -4344,7 +4344,7 @@
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B129" s="1">
         <v>11</v>
@@ -4361,7 +4361,7 @@
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B130" s="1">
         <v>7</v>
@@ -4378,7 +4378,7 @@
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B131" s="1">
         <v>10.5</v>
@@ -4395,7 +4395,7 @@
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B132" s="1">
         <v>8.5</v>
@@ -4412,7 +4412,7 @@
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B133" s="1">
         <v>11.5</v>
@@ -4429,7 +4429,7 @@
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B134" s="1">
         <v>9.5</v>
@@ -4446,7 +4446,7 @@
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B135" s="1">
         <v>9.5</v>
@@ -4463,7 +4463,7 @@
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B136" s="1">
         <v>7.5</v>
@@ -4480,7 +4480,7 @@
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B137" s="1">
         <v>11</v>
@@ -4497,7 +4497,7 @@
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B138" s="1">
         <v>11</v>
@@ -4514,7 +4514,7 @@
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B139" s="1">
         <v>8.5</v>
@@ -4531,7 +4531,7 @@
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B140" s="1">
         <v>11.5</v>
@@ -4548,7 +4548,7 @@
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B141" s="1">
         <v>11.5</v>
@@ -4565,7 +4565,7 @@
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B142" s="1">
         <v>7.5</v>
@@ -4582,7 +4582,7 @@
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B143" s="1">
         <v>10</v>
@@ -4599,7 +4599,7 @@
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B144" s="1">
         <v>10</v>
@@ -4616,7 +4616,7 @@
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B145" s="1">
         <v>10</v>
@@ -4633,7 +4633,7 @@
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B146" s="1">
         <v>7.5</v>
@@ -4650,7 +4650,7 @@
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B147" s="1">
         <v>8</v>
@@ -4667,7 +4667,7 @@
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B148" s="1">
         <v>9.5</v>
@@ -4684,7 +4684,7 @@
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B149" s="1">
         <v>7.5</v>
@@ -4701,7 +4701,7 @@
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B150" s="1">
         <v>9.5</v>
@@ -4718,7 +4718,7 @@
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B151" s="1">
         <v>12</v>
@@ -4735,7 +4735,7 @@
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B152" s="1">
         <v>11</v>
@@ -4752,7 +4752,7 @@
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B153" s="1">
         <v>10</v>
@@ -4769,7 +4769,7 @@
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B154" s="1">
         <v>10.5</v>
@@ -4786,7 +4786,7 @@
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B155" s="1">
         <v>10</v>
@@ -4803,7 +4803,7 @@
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B156" s="1">
         <v>6</v>
@@ -4820,7 +4820,7 @@
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B157" s="1">
         <v>8.5</v>
@@ -4837,7 +4837,7 @@
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B158" s="1">
         <v>10.5</v>
@@ -4854,7 +4854,7 @@
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B159" s="1">
         <v>10.5</v>
@@ -4871,7 +4871,7 @@
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B160" s="1">
         <v>10</v>
@@ -4888,7 +4888,7 @@
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B161" s="1">
         <v>11.5</v>
@@ -4905,7 +4905,7 @@
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B162" s="1">
         <v>10.5</v>
@@ -4922,7 +4922,7 @@
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B163" s="1">
         <v>11</v>
@@ -4939,7 +4939,7 @@
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B164" s="1">
         <v>8.5</v>
@@ -4956,7 +4956,7 @@
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B165" s="1">
         <v>8.5</v>
@@ -4973,7 +4973,7 @@
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B166" s="1">
         <v>10.5</v>
@@ -4990,7 +4990,7 @@
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B167" s="1">
         <v>10</v>
@@ -5007,7 +5007,7 @@
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B168" s="1">
         <v>11</v>
@@ -5024,7 +5024,7 @@
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B169" s="1">
         <v>12.5</v>
@@ -5041,7 +5041,7 @@
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B170" s="1">
         <v>9</v>
@@ -5058,7 +5058,7 @@
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B171" s="1">
         <v>9.5</v>
@@ -5075,7 +5075,7 @@
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B172" s="1">
         <v>9</v>
@@ -5092,7 +5092,7 @@
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B173" s="1">
         <v>6.5</v>
@@ -5109,7 +5109,7 @@
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B174" s="1">
         <v>7.5</v>
@@ -5126,7 +5126,7 @@
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B175" s="1">
         <v>9</v>
@@ -5143,7 +5143,7 @@
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B176" s="1">
         <v>10.5</v>
@@ -5160,7 +5160,7 @@
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B177" s="1">
         <v>8</v>
@@ -5177,7 +5177,7 @@
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B178" s="1">
         <v>9.5</v>
@@ -5194,7 +5194,7 @@
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B179" s="1">
         <v>11.5</v>
@@ -5211,7 +5211,7 @@
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B180" s="1">
         <v>6</v>
@@ -5228,7 +5228,7 @@
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B181" s="1">
         <v>13</v>
@@ -5245,7 +5245,7 @@
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B182" s="1">
         <v>8.5</v>
@@ -5262,7 +5262,7 @@
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B183" s="1">
         <v>7.5</v>
@@ -5279,7 +5279,7 @@
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B184" s="1">
         <v>11</v>
@@ -5296,7 +5296,7 @@
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B185" s="1">
         <v>8</v>
@@ -5313,7 +5313,7 @@
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B186" s="1">
         <v>8.5</v>
@@ -5330,7 +5330,7 @@
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B187" s="1">
         <v>9</v>
@@ -5347,7 +5347,7 @@
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B188" s="1">
         <v>11</v>
@@ -5364,7 +5364,7 @@
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B189" s="1">
         <v>6</v>
@@ -5381,7 +5381,7 @@
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B190" s="1">
         <v>6.5</v>
@@ -5398,7 +5398,7 @@
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B191" s="1">
         <v>9</v>
@@ -5415,7 +5415,7 @@
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B192" s="1">
         <v>9.5</v>
@@ -5432,7 +5432,7 @@
     </row>
     <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B193" s="1">
         <v>10</v>
@@ -5449,7 +5449,7 @@
     </row>
     <row r="194" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B194" s="1">
         <v>8.5</v>
@@ -5466,7 +5466,7 @@
     </row>
     <row r="195" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B195" s="1">
         <v>7</v>
@@ -5483,7 +5483,7 @@
     </row>
     <row r="196" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B196" s="1">
         <v>9</v>
@@ -5500,7 +5500,7 @@
     </row>
     <row r="197" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B197" s="1">
         <v>10.5</v>
@@ -5517,7 +5517,7 @@
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B198" s="1">
         <v>8.5</v>
@@ -5534,7 +5534,7 @@
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B199" s="1">
         <v>10</v>
@@ -5551,7 +5551,7 @@
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B200" s="1">
         <v>8</v>
@@ -5568,7 +5568,7 @@
     </row>
     <row r="201" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B201" s="1">
         <v>9.5</v>
@@ -5585,7 +5585,7 @@
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B202" s="1">
         <v>7</v>
@@ -5602,7 +5602,7 @@
     </row>
     <row r="203" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B203" s="1">
         <v>10</v>
@@ -5619,7 +5619,7 @@
     </row>
     <row r="204" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B204" s="1">
         <v>6.5</v>
@@ -5636,7 +5636,7 @@
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B205" s="1">
         <v>7.5</v>
@@ -5653,7 +5653,7 @@
     </row>
     <row r="206" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B206" s="1">
         <v>10</v>
@@ -5670,7 +5670,7 @@
     </row>
     <row r="207" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B207" s="1">
         <v>5.5</v>
@@ -5687,7 +5687,7 @@
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B208" s="1">
         <v>8</v>
@@ -5704,7 +5704,7 @@
     </row>
     <row r="209" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B209" s="1">
         <v>9.5</v>
@@ -5721,7 +5721,7 @@
     </row>
     <row r="210" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B210" s="1">
         <v>7</v>
@@ -5738,7 +5738,7 @@
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B211" s="1">
         <v>6.5</v>
@@ -5755,7 +5755,7 @@
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B212" s="1">
         <v>6.5</v>
@@ -5772,7 +5772,7 @@
     </row>
     <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B213" s="1">
         <v>9</v>
@@ -5789,7 +5789,7 @@
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B214" s="1">
         <v>10</v>
@@ -5806,7 +5806,7 @@
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B215" s="1">
         <v>9</v>
@@ -5823,7 +5823,7 @@
     </row>
     <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B216" s="1">
         <v>10</v>
@@ -5840,7 +5840,7 @@
     </row>
     <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B217" s="1">
         <v>8.5</v>
@@ -5857,7 +5857,7 @@
     </row>
     <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B218" s="1">
         <v>6</v>
@@ -5874,7 +5874,7 @@
     </row>
     <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B219" s="1">
         <v>5.5</v>
@@ -5891,7 +5891,7 @@
     </row>
     <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B220" s="1">
         <v>7.5</v>
@@ -5908,7 +5908,7 @@
     </row>
     <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B221" s="1">
         <v>8</v>
@@ -5925,7 +5925,7 @@
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B222" s="1">
         <v>7.5</v>
@@ -5942,7 +5942,7 @@
     </row>
     <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B223" s="1">
         <v>8.5</v>
@@ -5959,7 +5959,7 @@
     </row>
     <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B224" s="1">
         <v>11</v>
@@ -5976,7 +5976,7 @@
     </row>
     <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B225" s="1">
         <v>8.5</v>
@@ -5993,7 +5993,7 @@
     </row>
     <row r="226" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B226" s="1">
         <v>7</v>
@@ -6010,7 +6010,7 @@
     </row>
     <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B227" s="1">
         <v>11</v>
@@ -6027,7 +6027,7 @@
     </row>
     <row r="228" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B228" s="1">
         <v>8.5</v>
@@ -6044,7 +6044,7 @@
     </row>
     <row r="229" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B229" s="1">
         <v>9</v>
@@ -6061,7 +6061,7 @@
     </row>
     <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B230" s="1">
         <v>9</v>
@@ -6078,7 +6078,7 @@
     </row>
     <row r="231" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B231" s="1">
         <v>13</v>
@@ -6095,7 +6095,7 @@
     </row>
     <row r="232" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B232" s="1">
         <v>9.5</v>
@@ -6112,7 +6112,7 @@
     </row>
     <row r="233" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B233" s="1">
         <v>9.5</v>
@@ -6129,7 +6129,7 @@
     </row>
     <row r="234" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B234" s="1">
         <v>9.5</v>
@@ -6146,7 +6146,7 @@
     </row>
     <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B235" s="1">
         <v>12</v>
@@ -6163,7 +6163,7 @@
     </row>
     <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B236" s="1">
         <v>11</v>
@@ -6180,7 +6180,7 @@
     </row>
     <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B237" s="1">
         <v>7.5</v>
@@ -6197,7 +6197,7 @@
     </row>
     <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B238" s="1">
         <v>9</v>
@@ -6214,7 +6214,7 @@
     </row>
     <row r="239" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B239" s="1">
         <v>11</v>
@@ -6231,7 +6231,7 @@
     </row>
     <row r="240" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B240" s="1">
         <v>9.5</v>
@@ -6248,7 +6248,7 @@
     </row>
     <row r="241" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B241" s="1">
         <v>9.5</v>
@@ -6265,7 +6265,7 @@
     </row>
     <row r="242" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B242" s="1">
         <v>8.5</v>
@@ -6282,7 +6282,7 @@
     </row>
     <row r="243" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B243" s="1">
         <v>9</v>
@@ -6299,7 +6299,7 @@
     </row>
     <row r="244" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B244" s="1">
         <v>9</v>
@@ -6316,7 +6316,7 @@
     </row>
     <row r="245" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B245" s="1">
         <v>11</v>
@@ -6333,7 +6333,7 @@
     </row>
     <row r="246" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B246" s="1">
         <v>10.5</v>
@@ -6350,7 +6350,7 @@
     </row>
     <row r="247" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B247" s="1">
         <v>9</v>
@@ -6367,7 +6367,7 @@
     </row>
     <row r="248" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B248" s="1">
         <v>9.5</v>
@@ -6384,7 +6384,7 @@
     </row>
     <row r="249" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B249" s="1">
         <v>9</v>
@@ -6401,7 +6401,7 @@
     </row>
     <row r="250" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B250" s="1">
         <v>7</v>
@@ -6418,7 +6418,7 @@
     </row>
     <row r="251" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B251" s="1">
         <v>10</v>
@@ -6435,7 +6435,7 @@
     </row>
     <row r="252" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B252" s="1">
         <v>7.5</v>
@@ -6452,7 +6452,7 @@
     </row>
     <row r="253" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B253" s="1">
         <v>9</v>
@@ -6469,7 +6469,7 @@
     </row>
     <row r="254" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B254" s="1">
         <v>10</v>
@@ -6486,7 +6486,7 @@
     </row>
     <row r="255" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B255" s="1">
         <v>7.5</v>
@@ -6503,7 +6503,7 @@
     </row>
     <row r="256" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B256" s="1">
         <v>7.5</v>
@@ -6520,7 +6520,7 @@
     </row>
     <row r="257" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B257" s="1">
         <v>7.5</v>
@@ -6537,7 +6537,7 @@
     </row>
     <row r="258" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B258" s="1">
         <v>7</v>
@@ -6554,7 +6554,7 @@
     </row>
     <row r="259" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B259" s="1">
         <v>9</v>
@@ -6571,7 +6571,7 @@
     </row>
     <row r="260" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B260" s="1">
         <v>9.5</v>
@@ -6588,7 +6588,7 @@
     </row>
     <row r="261" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B261" s="1">
         <v>9.5</v>
@@ -6605,7 +6605,7 @@
     </row>
     <row r="262" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B262" s="1">
         <v>10</v>
@@ -6622,7 +6622,7 @@
     </row>
     <row r="263" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B263" s="1">
         <v>10.5</v>
@@ -6639,7 +6639,7 @@
     </row>
     <row r="264" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B264" s="1">
         <v>10.5</v>
@@ -6656,7 +6656,7 @@
     </row>
     <row r="265" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B265" s="1">
         <v>7.5</v>
@@ -6673,7 +6673,7 @@
     </row>
     <row r="266" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B266" s="1">
         <v>8</v>
@@ -6690,7 +6690,7 @@
     </row>
     <row r="267" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B267" s="1">
         <v>9.5</v>
@@ -6707,7 +6707,7 @@
     </row>
     <row r="268" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B268" s="1">
         <v>10.5</v>
@@ -6724,7 +6724,7 @@
     </row>
     <row r="269" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B269" s="1">
         <v>9.5</v>
@@ -6741,7 +6741,7 @@
     </row>
     <row r="270" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B270" s="1">
         <v>8</v>
@@ -6758,7 +6758,7 @@
     </row>
     <row r="271" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B271" s="1">
         <v>6.5</v>
@@ -6775,7 +6775,7 @@
     </row>
     <row r="272" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B272" s="1">
         <v>11</v>
@@ -6792,7 +6792,7 @@
     </row>
     <row r="273" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B273" s="1">
         <v>9.5</v>
@@ -6809,7 +6809,7 @@
     </row>
     <row r="274" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B274" s="1">
         <v>10</v>
@@ -6826,7 +6826,7 @@
     </row>
     <row r="275" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B275" s="1">
         <v>9</v>
@@ -6843,7 +6843,7 @@
     </row>
     <row r="276" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B276" s="1">
         <v>7.5</v>
@@ -6860,7 +6860,7 @@
     </row>
     <row r="277" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B277" s="1">
         <v>7.5</v>
@@ -6877,7 +6877,7 @@
     </row>
     <row r="278" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B278" s="1">
         <v>11.5</v>
@@ -6894,7 +6894,7 @@
     </row>
     <row r="279" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B279" s="1">
         <v>8</v>
@@ -6911,7 +6911,7 @@
     </row>
     <row r="280" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B280" s="1">
         <v>10.5</v>
@@ -6928,7 +6928,7 @@
     </row>
     <row r="281" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B281" s="1">
         <v>10.5</v>
@@ -6945,7 +6945,7 @@
     </row>
     <row r="282" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B282" s="1">
         <v>11.5</v>
@@ -6962,7 +6962,7 @@
     </row>
     <row r="283" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B283" s="1">
         <v>11</v>
@@ -6979,7 +6979,7 @@
     </row>
     <row r="284" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B284" s="1">
         <v>10</v>
@@ -6996,7 +6996,7 @@
     </row>
     <row r="285" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B285" s="1">
         <v>10</v>
@@ -7013,7 +7013,7 @@
     </row>
     <row r="286" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B286" s="1">
         <v>12</v>
@@ -7030,7 +7030,7 @@
     </row>
     <row r="287" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B287" s="1">
         <v>11.5</v>
@@ -7047,7 +7047,7 @@
     </row>
     <row r="288" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B288" s="1">
         <v>9.5</v>
@@ -7064,7 +7064,7 @@
     </row>
     <row r="289" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B289" s="1">
         <v>9.5</v>
@@ -7081,7 +7081,7 @@
     </row>
     <row r="290" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B290" s="1">
         <v>10.5</v>
@@ -7098,7 +7098,7 @@
     </row>
     <row r="291" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B291" s="1">
         <v>9.5</v>
@@ -7115,7 +7115,7 @@
     </row>
     <row r="292" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B292" s="1">
         <v>4.5</v>
@@ -7132,7 +7132,7 @@
     </row>
     <row r="293" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B293" s="1">
         <v>11.5</v>
@@ -7149,7 +7149,7 @@
     </row>
     <row r="294" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B294" s="1">
         <v>10.5</v>
@@ -7166,7 +7166,7 @@
     </row>
     <row r="295" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B295" s="1">
         <v>9.5</v>
@@ -7183,7 +7183,7 @@
     </row>
     <row r="296" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B296" s="1">
         <v>10</v>
@@ -7200,7 +7200,7 @@
     </row>
     <row r="297" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B297" s="1">
         <v>9</v>
@@ -7217,7 +7217,7 @@
     </row>
     <row r="298" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B298" s="1">
         <v>9</v>
@@ -7234,7 +7234,7 @@
     </row>
     <row r="299" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B299" s="1">
         <v>9</v>
@@ -7251,7 +7251,7 @@
     </row>
     <row r="300" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B300" s="1">
         <v>9</v>
@@ -7268,7 +7268,7 @@
     </row>
     <row r="301" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B301" s="1">
         <v>10.5</v>
@@ -7285,7 +7285,7 @@
     </row>
     <row r="302" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B302" s="1">
         <v>9</v>
@@ -7302,7 +7302,7 @@
     </row>
     <row r="303" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B303" s="1">
         <v>7</v>
@@ -7319,7 +7319,7 @@
     </row>
     <row r="304" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B304" s="1">
         <v>8.5</v>
@@ -7336,7 +7336,7 @@
     </row>
     <row r="305" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B305" s="1">
         <v>9.5</v>
@@ -7353,7 +7353,7 @@
     </row>
     <row r="306" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B306" s="1">
         <v>9</v>
@@ -7370,7 +7370,7 @@
     </row>
     <row r="307" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B307" s="1">
         <v>9</v>
@@ -7387,7 +7387,7 @@
     </row>
     <row r="308" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B308" s="1">
         <v>9</v>
@@ -7404,7 +7404,7 @@
     </row>
     <row r="309" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B309" s="1">
         <v>9</v>
@@ -7421,7 +7421,7 @@
     </row>
     <row r="310" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B310" s="1">
         <v>8.5</v>
@@ -7438,7 +7438,7 @@
     </row>
     <row r="311" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B311" s="1">
         <v>11.5</v>
@@ -7455,7 +7455,7 @@
     </row>
     <row r="312" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B312" s="1">
         <v>11</v>
@@ -7472,7 +7472,7 @@
     </row>
     <row r="313" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B313" s="1">
         <v>10.5</v>
@@ -7489,7 +7489,7 @@
     </row>
     <row r="314" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B314" s="1">
         <v>8</v>
@@ -7506,7 +7506,7 @@
     </row>
     <row r="315" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B315" s="1">
         <v>8</v>
@@ -7523,7 +7523,7 @@
     </row>
     <row r="316" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B316" s="1">
         <v>9.5</v>
@@ -7540,7 +7540,7 @@
     </row>
     <row r="317" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B317" s="1">
         <v>9.5</v>
@@ -7557,7 +7557,7 @@
     </row>
     <row r="318" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B318" s="1">
         <v>8.5</v>
@@ -7574,7 +7574,7 @@
     </row>
     <row r="319" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B319" s="1">
         <v>11</v>
@@ -7591,7 +7591,7 @@
     </row>
     <row r="320" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B320" s="1">
         <v>8</v>
@@ -7608,7 +7608,7 @@
     </row>
     <row r="321" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B321" s="1">
         <v>10</v>
@@ -7625,7 +7625,7 @@
     </row>
     <row r="322" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B322" s="1">
         <v>9</v>
@@ -7642,7 +7642,7 @@
     </row>
     <row r="323" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B323" s="1">
         <v>10</v>
@@ -7659,7 +7659,7 @@
     </row>
     <row r="324" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B324" s="1">
         <v>9.5</v>
@@ -7676,7 +7676,7 @@
     </row>
     <row r="325" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B325" s="1">
         <v>9</v>
@@ -7693,7 +7693,7 @@
     </row>
     <row r="326" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B326" s="1">
         <v>8</v>
@@ -7710,7 +7710,7 @@
     </row>
     <row r="327" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B327" s="1">
         <v>7.5</v>
@@ -7727,7 +7727,7 @@
     </row>
     <row r="328" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B328" s="1">
         <v>10</v>
@@ -7744,7 +7744,7 @@
     </row>
     <row r="329" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B329" s="1">
         <v>10</v>
@@ -7761,7 +7761,7 @@
     </row>
     <row r="330" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B330" s="1">
         <v>10.5</v>
@@ -7778,7 +7778,7 @@
     </row>
     <row r="331" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B331" s="1">
         <v>11.5</v>
@@ -7795,7 +7795,7 @@
     </row>
     <row r="332" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B332" s="1">
         <v>10.5</v>
@@ -7812,7 +7812,7 @@
     </row>
     <row r="333" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B333" s="1">
         <v>7.5</v>
@@ -7829,7 +7829,7 @@
     </row>
     <row r="334" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B334" s="1">
         <v>8</v>
@@ -7846,7 +7846,7 @@
     </row>
     <row r="335" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B335" s="1">
         <v>9.5</v>
@@ -7863,7 +7863,7 @@
     </row>
     <row r="336" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B336" s="1">
         <v>10</v>
@@ -7880,7 +7880,7 @@
     </row>
     <row r="337" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B337" s="1">
         <v>8.5</v>
@@ -7897,7 +7897,7 @@
     </row>
     <row r="338" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B338" s="1">
         <v>8.5</v>
@@ -7914,7 +7914,7 @@
     </row>
     <row r="339" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="B339" s="1">
         <v>9.5</v>
@@ -7931,7 +7931,7 @@
     </row>
     <row r="340" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B340" s="1">
         <v>11.5</v>
@@ -7948,7 +7948,7 @@
     </row>
     <row r="341" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B341" s="1">
         <v>10</v>
@@ -7965,7 +7965,7 @@
     </row>
     <row r="342" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B342" s="1">
         <v>10</v>
@@ -7982,7 +7982,7 @@
     </row>
     <row r="343" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B343" s="1">
         <v>9</v>
@@ -7999,7 +7999,7 @@
     </row>
     <row r="344" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B344" s="1">
         <v>8</v>
@@ -8016,7 +8016,7 @@
     </row>
     <row r="345" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B345" s="1">
         <v>12</v>
@@ -8033,7 +8033,7 @@
     </row>
     <row r="346" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B346" s="1">
         <v>8.5</v>
@@ -8050,7 +8050,7 @@
     </row>
     <row r="347" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B347" s="1">
         <v>9.5</v>
@@ -8067,7 +8067,7 @@
     </row>
     <row r="348" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B348" s="1">
         <v>10</v>
@@ -8084,7 +8084,7 @@
     </row>
     <row r="349" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B349" s="1">
         <v>10.5</v>
@@ -8101,7 +8101,7 @@
     </row>
     <row r="350" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B350" s="1">
         <v>9</v>
@@ -8118,7 +8118,7 @@
     </row>
     <row r="351" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B351" s="1">
         <v>11.5</v>
@@ -8135,7 +8135,7 @@
     </row>
     <row r="352" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B352" s="1">
         <v>7</v>
@@ -8152,7 +8152,7 @@
     </row>
     <row r="353" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B353" s="1">
         <v>10</v>
@@ -8169,7 +8169,7 @@
     </row>
     <row r="354" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B354" s="1">
         <v>10.5</v>
@@ -8186,7 +8186,7 @@
     </row>
     <row r="355" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B355" s="1">
         <v>9.5</v>
@@ -8203,7 +8203,7 @@
     </row>
     <row r="356" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B356" s="1">
         <v>8</v>
@@ -8220,7 +8220,7 @@
     </row>
     <row r="357" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B357" s="1">
         <v>13</v>
@@ -8237,7 +8237,7 @@
     </row>
     <row r="358" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B358" s="1">
         <v>9</v>
@@ -8254,7 +8254,7 @@
     </row>
     <row r="359" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B359" s="1">
         <v>9</v>
@@ -8271,7 +8271,7 @@
     </row>
     <row r="360" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B360" s="1">
         <v>9</v>
@@ -8288,7 +8288,7 @@
     </row>
     <row r="361" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B361" s="1">
         <v>6</v>
@@ -8305,7 +8305,7 @@
     </row>
     <row r="362" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B362" s="1">
         <v>10.5</v>
@@ -8322,7 +8322,7 @@
     </row>
     <row r="363" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B363" s="1">
         <v>9.5</v>
@@ -8339,7 +8339,7 @@
     </row>
     <row r="364" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B364" s="1">
         <v>8</v>
@@ -8356,7 +8356,7 @@
     </row>
     <row r="365" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B365" s="1">
         <v>8</v>
@@ -8373,7 +8373,7 @@
     </row>
     <row r="366" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B366" s="1">
         <v>10</v>
@@ -8390,7 +8390,7 @@
     </row>
     <row r="367" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B367" s="1">
         <v>7.5</v>
@@ -8407,7 +8407,7 @@
     </row>
     <row r="368" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B368" s="1">
         <v>10</v>
@@ -8424,7 +8424,7 @@
     </row>
     <row r="369" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B369" s="1">
         <v>10</v>
@@ -8441,7 +8441,7 @@
     </row>
     <row r="370" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B370" s="1">
         <v>7</v>
@@ -8458,7 +8458,7 @@
     </row>
     <row r="371" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B371" s="1">
         <v>9</v>
@@ -8475,7 +8475,7 @@
     </row>
     <row r="372" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B372" s="1">
         <v>10</v>
@@ -8492,7 +8492,7 @@
     </row>
     <row r="373" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B373" s="1">
         <v>8.5</v>
@@ -8509,7 +8509,7 @@
     </row>
     <row r="374" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B374" s="1">
         <v>11.5</v>
@@ -8526,7 +8526,7 @@
     </row>
     <row r="375" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B375" s="1">
         <v>9.5</v>
@@ -8543,7 +8543,7 @@
     </row>
     <row r="376" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B376" s="1">
         <v>10.5</v>
@@ -8560,7 +8560,7 @@
     </row>
     <row r="377" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B377" s="1">
         <v>12</v>
@@ -8577,7 +8577,7 @@
     </row>
     <row r="378" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B378" s="1">
         <v>10</v>
@@ -8594,7 +8594,7 @@
     </row>
     <row r="379" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B379" s="1">
         <v>10.5</v>
@@ -8611,7 +8611,7 @@
     </row>
     <row r="380" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="B380" s="1">
         <v>12</v>
@@ -8628,7 +8628,7 @@
     </row>
     <row r="381" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B381" s="1">
         <v>7.5</v>
@@ -8645,7 +8645,7 @@
     </row>
     <row r="382" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B382" s="1">
         <v>9.5</v>
@@ -8662,7 +8662,7 @@
     </row>
     <row r="383" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B383" s="1">
         <v>10</v>
@@ -8679,7 +8679,7 @@
     </row>
     <row r="384" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B384" s="1">
         <v>9</v>
@@ -8696,7 +8696,7 @@
     </row>
     <row r="385" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B385" s="1">
         <v>9.5</v>
@@ -8713,7 +8713,7 @@
     </row>
     <row r="386" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B386" s="1">
         <v>11</v>
@@ -8730,7 +8730,7 @@
     </row>
     <row r="387" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B387" s="1">
         <v>11</v>
@@ -8747,7 +8747,7 @@
     </row>
     <row r="388" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B388" s="1">
         <v>9</v>
@@ -8764,7 +8764,7 @@
     </row>
     <row r="389" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B389" s="1">
         <v>8.5</v>
@@ -8781,7 +8781,7 @@
     </row>
     <row r="390" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B390" s="1">
         <v>10</v>
@@ -8798,7 +8798,7 @@
     </row>
     <row r="391" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B391" s="1">
         <v>9.5</v>
@@ -8815,7 +8815,7 @@
     </row>
     <row r="392" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B392" s="1">
         <v>9</v>
@@ -8832,7 +8832,7 @@
     </row>
     <row r="393" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B393" s="1">
         <v>9</v>
@@ -8849,7 +8849,7 @@
     </row>
     <row r="394" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B394" s="1">
         <v>10</v>
@@ -8866,7 +8866,7 @@
     </row>
     <row r="395" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B395" s="1">
         <v>8</v>
@@ -8883,7 +8883,7 @@
     </row>
     <row r="396" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B396" s="1">
         <v>10</v>
@@ -8900,7 +8900,7 @@
     </row>
     <row r="397" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B397" s="1">
         <v>10.5</v>
@@ -8917,7 +8917,7 @@
     </row>
     <row r="398" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B398" s="1">
         <v>8.5</v>
@@ -8934,7 +8934,7 @@
     </row>
     <row r="399" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="B399" s="1">
         <v>10</v>
@@ -8951,7 +8951,7 @@
     </row>
     <row r="400" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B400" s="1">
         <v>9.5</v>
@@ -8968,7 +8968,7 @@
     </row>
     <row r="401" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B401" s="1">
         <v>11.5</v>
@@ -8985,7 +8985,7 @@
     </row>
     <row r="402" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B402" s="1">
         <v>8.5</v>
@@ -9002,7 +9002,7 @@
     </row>
     <row r="403" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B403" s="1">
         <v>10.5</v>
@@ -9019,7 +9019,7 @@
     </row>
     <row r="404" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B404" s="1">
         <v>9</v>
@@ -9036,7 +9036,7 @@
     </row>
     <row r="405" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B405" s="1">
         <v>10.5</v>
@@ -9053,7 +9053,7 @@
     </row>
     <row r="406" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B406" s="1">
         <v>10</v>
@@ -9070,7 +9070,7 @@
     </row>
     <row r="407" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B407" s="1">
         <v>10</v>
@@ -9087,7 +9087,7 @@
     </row>
     <row r="408" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B408" s="1">
         <v>10</v>
@@ -9104,7 +9104,7 @@
     </row>
     <row r="409" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B409" s="1">
         <v>10</v>
@@ -9121,7 +9121,7 @@
     </row>
     <row r="410" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B410" s="1">
         <v>10</v>
@@ -9138,7 +9138,7 @@
     </row>
     <row r="411" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B411" s="1">
         <v>11</v>
@@ -9155,7 +9155,7 @@
     </row>
     <row r="412" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B412" s="1">
         <v>9</v>
@@ -9172,7 +9172,7 @@
     </row>
     <row r="413" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B413" s="1">
         <v>10</v>
@@ -9189,7 +9189,7 @@
     </row>
     <row r="414" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B414" s="1">
         <v>9</v>
@@ -9206,7 +9206,7 @@
     </row>
     <row r="415" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B415" s="1">
         <v>10.5</v>
@@ -9223,7 +9223,7 @@
     </row>
     <row r="416" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B416" s="1">
         <v>11</v>
@@ -9240,7 +9240,7 @@
     </row>
     <row r="417" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B417" s="1">
         <v>9</v>
@@ -9257,7 +9257,7 @@
     </row>
     <row r="418" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B418" s="1">
         <v>9.5</v>
@@ -9274,7 +9274,7 @@
     </row>
     <row r="419" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B419" s="1">
         <v>10.5</v>
@@ -9291,7 +9291,7 @@
     </row>
     <row r="420" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B420" s="1">
         <v>10</v>
@@ -9308,7 +9308,7 @@
     </row>
     <row r="421" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B421" s="1">
         <v>10</v>

</xml_diff>